<commit_message>
Minor fixes. Fixed scoreboard bug (fname). Updated heart printing line from '\t' to '  '.
</commit_message>
<xml_diff>
--- a/data/artikel.xlsx
+++ b/data/artikel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jwt/Documents/Code/gelato/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A26A6D-97B3-A440-B133-E48FBF042B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15A22D8-8FF1-BB4C-9E1C-C458B4ABDE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1720" yWindow="2820" windowWidth="21820" windowHeight="14180" xr2:uid="{2D6BCF81-A2D9-5B4D-AD53-B365A8194329}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{2D6BCF81-A2D9-5B4D-AD53-B365A8194329}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="171">
   <si>
     <t>Artikel</t>
   </si>
@@ -281,9 +281,6 @@
     <t>Salsa</t>
   </si>
   <si>
-    <t>Ketchup</t>
-  </si>
-  <si>
     <t>Senf</t>
   </si>
   <si>
@@ -480,12 +477,6 @@
   </si>
   <si>
     <t>Handlebar</t>
-  </si>
-  <si>
-    <t>Bremsen</t>
-  </si>
-  <si>
-    <t>Brakes</t>
   </si>
   <si>
     <t>Schalthebel</t>
@@ -597,7 +588,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -613,9 +604,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -653,7 +644,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -759,7 +750,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -901,7 +892,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -909,7 +900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67AD30F3-BC96-AA4E-AB81-F5562BDF30AC}">
-  <dimension ref="A1:D83"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -942,7 +933,7 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -956,7 +947,7 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -970,7 +961,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -984,7 +975,7 @@
         <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -998,7 +989,7 @@
         <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -1012,7 +1003,7 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1026,7 +1017,7 @@
         <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -1040,7 +1031,7 @@
         <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -1054,7 +1045,7 @@
         <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -1068,7 +1059,7 @@
         <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -1096,7 +1087,7 @@
         <v>28</v>
       </c>
       <c r="D13" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -1146,10 +1137,10 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
+        <v>137</v>
+      </c>
+      <c r="C17" t="s">
         <v>138</v>
-      </c>
-      <c r="C17" t="s">
-        <v>139</v>
       </c>
       <c r="D17" t="s">
         <v>66</v>
@@ -1359,7 +1350,7 @@
         <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D32" t="s">
         <v>65</v>
@@ -1373,7 +1364,7 @@
         <v>68</v>
       </c>
       <c r="C33" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D33" t="s">
         <v>65</v>
@@ -1387,7 +1378,7 @@
         <v>69</v>
       </c>
       <c r="C34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D34" t="s">
         <v>65</v>
@@ -1401,7 +1392,7 @@
         <v>70</v>
       </c>
       <c r="C35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D35" t="s">
         <v>65</v>
@@ -1429,7 +1420,7 @@
         <v>73</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D37" t="s">
         <v>65</v>
@@ -1443,7 +1434,7 @@
         <v>74</v>
       </c>
       <c r="C38" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D38" t="s">
         <v>65</v>
@@ -1457,7 +1448,7 @@
         <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D39" t="s">
         <v>65</v>
@@ -1471,7 +1462,7 @@
         <v>72</v>
       </c>
       <c r="C40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D40" t="s">
         <v>76</v>
@@ -1485,7 +1476,7 @@
         <v>77</v>
       </c>
       <c r="C41" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D41" t="s">
         <v>76</v>
@@ -1499,7 +1490,7 @@
         <v>78</v>
       </c>
       <c r="C42" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D42" t="s">
         <v>76</v>
@@ -1513,7 +1504,7 @@
         <v>79</v>
       </c>
       <c r="C43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D43" t="s">
         <v>76</v>
@@ -1524,7 +1515,7 @@
         <v>25</v>
       </c>
       <c r="B44" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C44" t="s">
         <v>80</v>
@@ -1535,13 +1526,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B45" t="s">
         <v>81</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="D45" t="s">
         <v>76</v>
@@ -1549,13 +1540,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B46" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C46" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D46" t="s">
         <v>76</v>
@@ -1563,10 +1554,10 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B47" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C47" t="s">
         <v>96</v>
@@ -1580,55 +1571,55 @@
         <v>25</v>
       </c>
       <c r="B48" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="C48" t="s">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="D48" t="s">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B49" t="s">
-        <v>84</v>
+        <v>118</v>
       </c>
       <c r="C49" t="s">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="D49" t="s">
-        <v>76</v>
+        <v>116</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B50" t="s">
         <v>98</v>
       </c>
       <c r="C50" t="s">
+        <v>117</v>
+      </c>
+      <c r="D50" t="s">
         <v>116</v>
-      </c>
-      <c r="D50" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B51" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="C51" t="s">
         <v>120</v>
       </c>
       <c r="D51" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
@@ -1636,27 +1627,27 @@
         <v>22</v>
       </c>
       <c r="B52" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C52" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D52" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="B53" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C53" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D53" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
@@ -1664,27 +1655,27 @@
         <v>22</v>
       </c>
       <c r="B54" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C54" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D54" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B55" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C55" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D55" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
@@ -1692,13 +1683,13 @@
         <v>22</v>
       </c>
       <c r="B56" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C56" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D56" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
@@ -1706,13 +1697,13 @@
         <v>22</v>
       </c>
       <c r="B57" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C57" t="s">
         <v>125</v>
       </c>
       <c r="D57" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
@@ -1720,13 +1711,13 @@
         <v>22</v>
       </c>
       <c r="B58" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C58" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D58" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
@@ -1734,13 +1725,13 @@
         <v>22</v>
       </c>
       <c r="B59" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C59" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D59" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
@@ -1748,27 +1739,27 @@
         <v>22</v>
       </c>
       <c r="B60" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C60" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D60" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B61" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C61" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
@@ -1776,41 +1767,41 @@
         <v>22</v>
       </c>
       <c r="B62" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C62" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D62" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B63" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C63" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D63" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B64" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C64" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D64" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -1818,13 +1809,13 @@
         <v>22</v>
       </c>
       <c r="B65" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C65" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D65" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -1832,13 +1823,13 @@
         <v>25</v>
       </c>
       <c r="B66" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C66" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D66" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -1846,13 +1837,13 @@
         <v>22</v>
       </c>
       <c r="B67" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="C67" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D67" t="s">
-        <v>117</v>
+        <v>163</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
@@ -1860,55 +1851,55 @@
         <v>25</v>
       </c>
       <c r="B68" t="s">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="C68" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D68" t="s">
-        <v>117</v>
+        <v>163</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B69" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C69" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D69" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B70" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C70" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D70" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B71" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C71" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D71" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
@@ -1916,69 +1907,69 @@
         <v>22</v>
       </c>
       <c r="B72" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="C72" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D72" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B73" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="C73" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D73" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B74" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="C74" t="s">
         <v>151</v>
       </c>
       <c r="D74" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B75" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
       <c r="C75" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D75" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B76" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="C76" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D76" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
@@ -1986,13 +1977,13 @@
         <v>25</v>
       </c>
       <c r="B77" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="C77" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D77" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
@@ -2000,27 +1991,27 @@
         <v>25</v>
       </c>
       <c r="B78" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="C78" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D78" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B79" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C79" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D79" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
@@ -2028,55 +2019,13 @@
         <v>25</v>
       </c>
       <c r="B80" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C80" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D80" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>25</v>
-      </c>
-      <c r="B81" t="s">
-        <v>170</v>
-      </c>
-      <c r="C81" t="s">
-        <v>161</v>
-      </c>
-      <c r="D81" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>22</v>
-      </c>
-      <c r="B82" t="s">
-        <v>162</v>
-      </c>
-      <c r="C82" t="s">
         <v>163</v>
-      </c>
-      <c r="D82" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>25</v>
-      </c>
-      <c r="B83" t="s">
-        <v>164</v>
-      </c>
-      <c r="C83" t="s">
-        <v>165</v>
-      </c>
-      <c r="D83" t="s">
-        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated first page of the documentation.
</commit_message>
<xml_diff>
--- a/data/artikel.xlsx
+++ b/data/artikel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jwt/Documents/Code/gelato/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15A22D8-8FF1-BB4C-9E1C-C458B4ABDE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5F1B7C-2F7E-794A-8CA8-9C8EF10C7CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{2D6BCF81-A2D9-5B4D-AD53-B365A8194329}"/>
+    <workbookView xWindow="4520" yWindow="960" windowWidth="33940" windowHeight="18980" xr2:uid="{2D6BCF81-A2D9-5B4D-AD53-B365A8194329}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="265">
   <si>
     <t>Artikel</t>
   </si>
@@ -549,6 +549,288 @@
   </si>
   <si>
     <t>Salsa (Soßen)</t>
+  </si>
+  <si>
+    <t>Erdbeere</t>
+  </si>
+  <si>
+    <t>Strawberry</t>
+  </si>
+  <si>
+    <t>Apfel</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Aprikose</t>
+  </si>
+  <si>
+    <t>Apricot</t>
+  </si>
+  <si>
+    <t>Pfirsich</t>
+  </si>
+  <si>
+    <t>Nektarine</t>
+  </si>
+  <si>
+    <t>Pflaume</t>
+  </si>
+  <si>
+    <t>Birne</t>
+  </si>
+  <si>
+    <t>Grapefruit</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Zitrone</t>
+  </si>
+  <si>
+    <t>Limette</t>
+  </si>
+  <si>
+    <t>Banane</t>
+  </si>
+  <si>
+    <t>Wassermelone</t>
+  </si>
+  <si>
+    <t>Schnitz</t>
+  </si>
+  <si>
+    <t>Schale</t>
+  </si>
+  <si>
+    <t>Obst</t>
+  </si>
+  <si>
+    <t>Weizenmehl</t>
+  </si>
+  <si>
+    <t>Croissant</t>
+  </si>
+  <si>
+    <t>Weissbrot</t>
+  </si>
+  <si>
+    <t>Sandwich</t>
+  </si>
+  <si>
+    <t>Tortilla</t>
+  </si>
+  <si>
+    <t>Bagel</t>
+  </si>
+  <si>
+    <t>Scheibe</t>
+  </si>
+  <si>
+    <t>Brot</t>
+  </si>
+  <si>
+    <t>Kopf</t>
+  </si>
+  <si>
+    <t>Brustkorb</t>
+  </si>
+  <si>
+    <t>Arm</t>
+  </si>
+  <si>
+    <t>Bauch</t>
+  </si>
+  <si>
+    <t>Hüfte</t>
+  </si>
+  <si>
+    <t>Leiste</t>
+  </si>
+  <si>
+    <t>Oberschenkel</t>
+  </si>
+  <si>
+    <t>Knie</t>
+  </si>
+  <si>
+    <t>Schienbein</t>
+  </si>
+  <si>
+    <t>Hals</t>
+  </si>
+  <si>
+    <t>Schulter</t>
+  </si>
+  <si>
+    <t>Brust</t>
+  </si>
+  <si>
+    <t>Schamgegend</t>
+  </si>
+  <si>
+    <t>Bein</t>
+  </si>
+  <si>
+    <t>Fuß</t>
+  </si>
+  <si>
+    <t>Nacken</t>
+  </si>
+  <si>
+    <t>Schulterblatt</t>
+  </si>
+  <si>
+    <t>Taille</t>
+  </si>
+  <si>
+    <t>Gesäß</t>
+  </si>
+  <si>
+    <t>Kniekehle</t>
+  </si>
+  <si>
+    <t>Ferse</t>
+  </si>
+  <si>
+    <t>Ellbogen</t>
+  </si>
+  <si>
+    <t>Rücken</t>
+  </si>
+  <si>
+    <t>Handgelenk</t>
+  </si>
+  <si>
+    <t>Wade</t>
+  </si>
+  <si>
+    <t>Knöchel</t>
+  </si>
+  <si>
+    <t>Körper</t>
+  </si>
+  <si>
+    <t>Peach</t>
+  </si>
+  <si>
+    <t>Nectarine</t>
+  </si>
+  <si>
+    <t>Plum</t>
+  </si>
+  <si>
+    <t>Pear</t>
+  </si>
+  <si>
+    <t>orange</t>
+  </si>
+  <si>
+    <t>Lemon</t>
+  </si>
+  <si>
+    <t>Lime</t>
+  </si>
+  <si>
+    <t>Banana</t>
+  </si>
+  <si>
+    <t>Watermelon</t>
+  </si>
+  <si>
+    <t>Peel</t>
+  </si>
+  <si>
+    <t>slice</t>
+  </si>
+  <si>
+    <t>Wheat flour</t>
+  </si>
+  <si>
+    <t>White bread</t>
+  </si>
+  <si>
+    <t>sandwich</t>
+  </si>
+  <si>
+    <t>bagel</t>
+  </si>
+  <si>
+    <t>Slice of bread</t>
+  </si>
+  <si>
+    <t>Head</t>
+  </si>
+  <si>
+    <t>Brisket</t>
+  </si>
+  <si>
+    <t>Belly</t>
+  </si>
+  <si>
+    <t>Hip</t>
+  </si>
+  <si>
+    <t>Groin</t>
+  </si>
+  <si>
+    <t>Thigh</t>
+  </si>
+  <si>
+    <t>Knee</t>
+  </si>
+  <si>
+    <t>Shin</t>
+  </si>
+  <si>
+    <t>Neck</t>
+  </si>
+  <si>
+    <t>Shoulder</t>
+  </si>
+  <si>
+    <t>Chest</t>
+  </si>
+  <si>
+    <t>Pubic area</t>
+  </si>
+  <si>
+    <t>Leg</t>
+  </si>
+  <si>
+    <t>Foot</t>
+  </si>
+  <si>
+    <t>Shoulder blade</t>
+  </si>
+  <si>
+    <t>Waist</t>
+  </si>
+  <si>
+    <t>Buttocks</t>
+  </si>
+  <si>
+    <t>Back of the knee</t>
+  </si>
+  <si>
+    <t>Heel</t>
+  </si>
+  <si>
+    <t>Elbow</t>
+  </si>
+  <si>
+    <t>back</t>
+  </si>
+  <si>
+    <t>Wrist</t>
+  </si>
+  <si>
+    <t>Calf</t>
+  </si>
+  <si>
+    <t>Ankle</t>
   </si>
 </sst>
 </file>
@@ -900,7 +1182,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67AD30F3-BC96-AA4E-AB81-F5562BDF30AC}">
-  <dimension ref="A1:D80"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -2028,6 +2310,692 @@
         <v>163</v>
       </c>
     </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>4</v>
+      </c>
+      <c r="B81" t="s">
+        <v>171</v>
+      </c>
+      <c r="C81" t="s">
+        <v>172</v>
+      </c>
+      <c r="D81" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>22</v>
+      </c>
+      <c r="B82" t="s">
+        <v>173</v>
+      </c>
+      <c r="C82" t="s">
+        <v>174</v>
+      </c>
+      <c r="D82" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>25</v>
+      </c>
+      <c r="B83" t="s">
+        <v>175</v>
+      </c>
+      <c r="C83" t="s">
+        <v>176</v>
+      </c>
+      <c r="D83" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>22</v>
+      </c>
+      <c r="B84" t="s">
+        <v>177</v>
+      </c>
+      <c r="C84" t="s">
+        <v>225</v>
+      </c>
+      <c r="D84" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>25</v>
+      </c>
+      <c r="B85" t="s">
+        <v>178</v>
+      </c>
+      <c r="C85" t="s">
+        <v>226</v>
+      </c>
+      <c r="D85" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>25</v>
+      </c>
+      <c r="B86" t="s">
+        <v>179</v>
+      </c>
+      <c r="C86" t="s">
+        <v>227</v>
+      </c>
+      <c r="D86" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>25</v>
+      </c>
+      <c r="B87" t="s">
+        <v>180</v>
+      </c>
+      <c r="C87" t="s">
+        <v>228</v>
+      </c>
+      <c r="D87" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>25</v>
+      </c>
+      <c r="B88" t="s">
+        <v>181</v>
+      </c>
+      <c r="C88" t="s">
+        <v>181</v>
+      </c>
+      <c r="D88" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>25</v>
+      </c>
+      <c r="B89" t="s">
+        <v>182</v>
+      </c>
+      <c r="C89" t="s">
+        <v>229</v>
+      </c>
+      <c r="D89" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>25</v>
+      </c>
+      <c r="B90" t="s">
+        <v>183</v>
+      </c>
+      <c r="C90" t="s">
+        <v>230</v>
+      </c>
+      <c r="D90" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>25</v>
+      </c>
+      <c r="B91" t="s">
+        <v>184</v>
+      </c>
+      <c r="C91" t="s">
+        <v>231</v>
+      </c>
+      <c r="D91" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>25</v>
+      </c>
+      <c r="B92" t="s">
+        <v>185</v>
+      </c>
+      <c r="C92" t="s">
+        <v>232</v>
+      </c>
+      <c r="D92" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>25</v>
+      </c>
+      <c r="B93" t="s">
+        <v>186</v>
+      </c>
+      <c r="C93" t="s">
+        <v>233</v>
+      </c>
+      <c r="D93" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>25</v>
+      </c>
+      <c r="B94" t="s">
+        <v>188</v>
+      </c>
+      <c r="C94" t="s">
+        <v>234</v>
+      </c>
+      <c r="D94" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>22</v>
+      </c>
+      <c r="B95" t="s">
+        <v>187</v>
+      </c>
+      <c r="C95" t="s">
+        <v>235</v>
+      </c>
+      <c r="D95" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>2</v>
+      </c>
+      <c r="B96" t="s">
+        <v>190</v>
+      </c>
+      <c r="C96" t="s">
+        <v>236</v>
+      </c>
+      <c r="D96" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>2</v>
+      </c>
+      <c r="B97" t="s">
+        <v>191</v>
+      </c>
+      <c r="C97" t="s">
+        <v>191</v>
+      </c>
+      <c r="D97" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>2</v>
+      </c>
+      <c r="B98" t="s">
+        <v>192</v>
+      </c>
+      <c r="C98" t="s">
+        <v>237</v>
+      </c>
+      <c r="D98" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>2</v>
+      </c>
+      <c r="B99" t="s">
+        <v>193</v>
+      </c>
+      <c r="C99" t="s">
+        <v>238</v>
+      </c>
+      <c r="D99" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>25</v>
+      </c>
+      <c r="B100" t="s">
+        <v>194</v>
+      </c>
+      <c r="C100" t="s">
+        <v>194</v>
+      </c>
+      <c r="D100" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>22</v>
+      </c>
+      <c r="B101" t="s">
+        <v>195</v>
+      </c>
+      <c r="C101" t="s">
+        <v>239</v>
+      </c>
+      <c r="D101" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>25</v>
+      </c>
+      <c r="B102" t="s">
+        <v>196</v>
+      </c>
+      <c r="C102" t="s">
+        <v>240</v>
+      </c>
+      <c r="D102" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>22</v>
+      </c>
+      <c r="B103" t="s">
+        <v>198</v>
+      </c>
+      <c r="C103" t="s">
+        <v>241</v>
+      </c>
+      <c r="D103" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>22</v>
+      </c>
+      <c r="B104" t="s">
+        <v>199</v>
+      </c>
+      <c r="C104" t="s">
+        <v>242</v>
+      </c>
+      <c r="D104" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>22</v>
+      </c>
+      <c r="B105" t="s">
+        <v>200</v>
+      </c>
+      <c r="C105" t="s">
+        <v>200</v>
+      </c>
+      <c r="D105" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>22</v>
+      </c>
+      <c r="B106" t="s">
+        <v>201</v>
+      </c>
+      <c r="C106" t="s">
+        <v>243</v>
+      </c>
+      <c r="D106" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>25</v>
+      </c>
+      <c r="B107" t="s">
+        <v>202</v>
+      </c>
+      <c r="C107" t="s">
+        <v>244</v>
+      </c>
+      <c r="D107" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>25</v>
+      </c>
+      <c r="B108" t="s">
+        <v>203</v>
+      </c>
+      <c r="C108" t="s">
+        <v>245</v>
+      </c>
+      <c r="D108" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>22</v>
+      </c>
+      <c r="B109" t="s">
+        <v>204</v>
+      </c>
+      <c r="C109" t="s">
+        <v>246</v>
+      </c>
+      <c r="D109" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>2</v>
+      </c>
+      <c r="B110" t="s">
+        <v>205</v>
+      </c>
+      <c r="C110" t="s">
+        <v>247</v>
+      </c>
+      <c r="D110" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>2</v>
+      </c>
+      <c r="B111" t="s">
+        <v>206</v>
+      </c>
+      <c r="C111" t="s">
+        <v>248</v>
+      </c>
+      <c r="D111" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>22</v>
+      </c>
+      <c r="B112" t="s">
+        <v>207</v>
+      </c>
+      <c r="C112" t="s">
+        <v>249</v>
+      </c>
+      <c r="D112" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>25</v>
+      </c>
+      <c r="B113" t="s">
+        <v>208</v>
+      </c>
+      <c r="C113" t="s">
+        <v>250</v>
+      </c>
+      <c r="D113" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>25</v>
+      </c>
+      <c r="B114" t="s">
+        <v>209</v>
+      </c>
+      <c r="C114" t="s">
+        <v>251</v>
+      </c>
+      <c r="D114" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>25</v>
+      </c>
+      <c r="B115" t="s">
+        <v>210</v>
+      </c>
+      <c r="C115" t="s">
+        <v>252</v>
+      </c>
+      <c r="D115" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>2</v>
+      </c>
+      <c r="B116" t="s">
+        <v>211</v>
+      </c>
+      <c r="C116" t="s">
+        <v>253</v>
+      </c>
+      <c r="D116" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>22</v>
+      </c>
+      <c r="B117" t="s">
+        <v>212</v>
+      </c>
+      <c r="C117" t="s">
+        <v>254</v>
+      </c>
+      <c r="D117" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>22</v>
+      </c>
+      <c r="B118" t="s">
+        <v>213</v>
+      </c>
+      <c r="C118" t="s">
+        <v>249</v>
+      </c>
+      <c r="D118" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>2</v>
+      </c>
+      <c r="B119" t="s">
+        <v>214</v>
+      </c>
+      <c r="C119" t="s">
+        <v>255</v>
+      </c>
+      <c r="D119" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>25</v>
+      </c>
+      <c r="B120" t="s">
+        <v>215</v>
+      </c>
+      <c r="C120" t="s">
+        <v>256</v>
+      </c>
+      <c r="D120" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>2</v>
+      </c>
+      <c r="B121" t="s">
+        <v>216</v>
+      </c>
+      <c r="C121" t="s">
+        <v>257</v>
+      </c>
+      <c r="D121" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>25</v>
+      </c>
+      <c r="B122" t="s">
+        <v>217</v>
+      </c>
+      <c r="C122" t="s">
+        <v>258</v>
+      </c>
+      <c r="D122" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>25</v>
+      </c>
+      <c r="B123" t="s">
+        <v>218</v>
+      </c>
+      <c r="C123" t="s">
+        <v>259</v>
+      </c>
+      <c r="D123" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>22</v>
+      </c>
+      <c r="B124" t="s">
+        <v>219</v>
+      </c>
+      <c r="C124" t="s">
+        <v>260</v>
+      </c>
+      <c r="D124" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>22</v>
+      </c>
+      <c r="B125" t="s">
+        <v>220</v>
+      </c>
+      <c r="C125" t="s">
+        <v>261</v>
+      </c>
+      <c r="D125" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>2</v>
+      </c>
+      <c r="B126" t="s">
+        <v>221</v>
+      </c>
+      <c r="C126" t="s">
+        <v>262</v>
+      </c>
+      <c r="D126" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>25</v>
+      </c>
+      <c r="B127" t="s">
+        <v>221</v>
+      </c>
+      <c r="C127" t="s">
+        <v>262</v>
+      </c>
+      <c r="D127" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>4</v>
+      </c>
+      <c r="B128" t="s">
+        <v>222</v>
+      </c>
+      <c r="C128" t="s">
+        <v>263</v>
+      </c>
+      <c r="D128" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
+        <v>22</v>
+      </c>
+      <c r="B129" t="s">
+        <v>223</v>
+      </c>
+      <c r="C129" t="s">
+        <v>264</v>
+      </c>
+      <c r="D129" t="s">
+        <v>224</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>